<commit_message>
fix en index export
</commit_message>
<xml_diff>
--- a/publishing/accessibility/springer_alt_text_inventory.xlsx
+++ b/publishing/accessibility/springer_alt_text_inventory.xlsx
@@ -662,16 +662,18 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Front-Matter Guide: Publication Structure and Reading Paths</t>
+          <t>Preface</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>docs/en/front_matter_guide.md</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="n">
-        <v>7</v>
+          <t>docs/en/preface.md</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="H3" s="15" t="n"/>
       <c r="I3" s="8" t="inlineStr">
@@ -16937,7 +16939,7 @@
       </c>
       <c r="K212" s="8" t="inlineStr">
         <is>
-          <t>docs/images/part14/Yu-Project13-Fig02-EN.svg</t>
+          <t>docs/images/part14/Yu-Project13-Fig01-EN.svg</t>
         </is>
       </c>
       <c r="L212" s="8" t="inlineStr">

</xml_diff>

<commit_message>
fix zh/en export Edition Status
</commit_message>
<xml_diff>
--- a/publishing/accessibility/springer_alt_text_inventory.xlsx
+++ b/publishing/accessibility/springer_alt_text_inventory.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AltText" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AltText" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -4973,7 +4973,11 @@
           <t>jpg</t>
         </is>
       </c>
-      <c r="O60" s="17" t="n"/>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Second panel of a shark attack infographic summarizing state-level shark attacks in the United States over the past ten years, with Florida and Hawaii showing the largest totals.</t>
+        </is>
+      </c>
       <c r="P60" s="8" t="n"/>
     </row>
     <row r="61" ht="98" customHeight="1" s="6">
@@ -5041,7 +5045,11 @@
           <t>jpg</t>
         </is>
       </c>
-      <c r="O61" s="17" t="n"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Third panel of a shark attack infographic showing a 2013-2022 timeline matrix by state, including yearly attack counts and fatal incident markers.</t>
+        </is>
+      </c>
       <c r="P61" s="8" t="n"/>
     </row>
     <row r="62" ht="84" customHeight="1" s="6">
@@ -5109,7 +5117,11 @@
           <t>jpg</t>
         </is>
       </c>
-      <c r="O62" s="18" t="n"/>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Fourth panel of a shark attack infographic comparing average annual shark deaths with other accidental-death risks such as falls, deer collisions, bees, lightning, dogs, cows, snakes, and vending machines.</t>
+        </is>
+      </c>
       <c r="P62" s="8" t="n"/>
     </row>
     <row r="63" ht="70" customHeight="1" s="6">
@@ -23007,9 +23019,6 @@
       <c r="P293" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="O59:O62"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>